<commit_message>
Update /output from Ganymede2 run
</commit_message>
<xml_diff>
--- a/phys5v48hw/hw4/output/asyncLorentz/asyncLorentzCat.xlsx
+++ b/phys5v48hw/hw4/output/asyncLorentz/asyncLorentzCat.xlsx
@@ -1,52 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <workbookPr codeName="ThisWorkbook"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
+  <workbookProtection/>
+  <bookViews>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+  </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
   <fonts count="1">
     <font>
-      <sz val="12"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -65,13 +47,80 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -150,7 +199,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -185,7 +233,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -220,16 +267,20 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="100000"/>
-                <a:shade val="100000"/>
+                <a:shade val="51000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-                <a:shade val="100000"/>
-                <a:satMod val="350000"/>
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -351,80 +402,448 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults>
-    <a:spDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="3">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="lt1"/>
-        </a:fontRef>
-      </a:style>
-    </a:spDef>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
+  <a:objectDefaults/>
   <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="B1:H1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" t="str">
-        <v>Problem Size (n)</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Bins</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Nodes</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Ranks</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Threads Per Rank</v>
-      </c>
-      <c r="G1" t="str">
-        <v>Runtime</v>
-      </c>
-      <c r="H1" t="str">
-        <v>Peak Memory</v>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Problem Size (n)</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Bins</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Nodes</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Ranks</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Threads Per Rank</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Runtime</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Peak Memory</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>0</v>
+      </c>
+      <c r="B2" t="n">
+        <v>100000000</v>
+      </c>
+      <c r="C2" t="n">
+        <v>10</v>
+      </c>
+      <c r="D2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G2" t="n">
+        <v>1.529987089335918</v>
+      </c>
+      <c r="H2" t="n">
+        <v>140824</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="n">
+        <v>100000000</v>
+      </c>
+      <c r="C3" t="n">
+        <v>100</v>
+      </c>
+      <c r="D3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G3" t="n">
+        <v>1.444251174107194</v>
+      </c>
+      <c r="H3" t="n">
+        <v>141060</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" t="n">
+        <v>100000000</v>
+      </c>
+      <c r="C4" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G4" t="n">
+        <v>1.459728951565921</v>
+      </c>
+      <c r="H4" t="n">
+        <v>140796</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" t="n">
+        <v>100000000</v>
+      </c>
+      <c r="C5" t="n">
+        <v>10</v>
+      </c>
+      <c r="D5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" t="n">
+        <v>1.48496988043189</v>
+      </c>
+      <c r="H5" t="n">
+        <v>140820</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" t="n">
+        <v>100000000</v>
+      </c>
+      <c r="C6" t="n">
+        <v>100</v>
+      </c>
+      <c r="D6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" t="n">
+        <v>1.447627434507012</v>
+      </c>
+      <c r="H6" t="n">
+        <v>141332</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" t="n">
+        <v>100000000</v>
+      </c>
+      <c r="C7" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" t="n">
+        <v>1.430273515172303</v>
+      </c>
+      <c r="H7" t="n">
+        <v>141116</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" t="n">
+        <v>100000000</v>
+      </c>
+      <c r="C8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E8" t="n">
+        <v>4</v>
+      </c>
+      <c r="F8" t="n">
+        <v>2</v>
+      </c>
+      <c r="G8" t="n">
+        <v>1.468488277867436</v>
+      </c>
+      <c r="H8" t="n">
+        <v>140492</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" t="n">
+        <v>100000000</v>
+      </c>
+      <c r="C9" t="n">
+        <v>100</v>
+      </c>
+      <c r="D9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E9" t="n">
+        <v>4</v>
+      </c>
+      <c r="F9" t="n">
+        <v>2</v>
+      </c>
+      <c r="G9" t="n">
+        <v>1.430536544881761</v>
+      </c>
+      <c r="H9" t="n">
+        <v>140544</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" t="n">
+        <v>100000000</v>
+      </c>
+      <c r="C10" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D10" t="n">
+        <v>2</v>
+      </c>
+      <c r="E10" t="n">
+        <v>4</v>
+      </c>
+      <c r="F10" t="n">
+        <v>2</v>
+      </c>
+      <c r="G10" t="n">
+        <v>1.455748470500112</v>
+      </c>
+      <c r="H10" t="n">
+        <v>141056</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" t="n">
+        <v>100000000</v>
+      </c>
+      <c r="C11" t="n">
+        <v>10</v>
+      </c>
+      <c r="D11" t="n">
+        <v>2</v>
+      </c>
+      <c r="E11" t="n">
+        <v>8</v>
+      </c>
+      <c r="F11" t="n">
+        <v>4</v>
+      </c>
+      <c r="G11" t="n">
+        <v>1.470564786344767</v>
+      </c>
+      <c r="H11" t="n">
+        <v>141084</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" t="n">
+        <v>100000000</v>
+      </c>
+      <c r="C12" t="n">
+        <v>100</v>
+      </c>
+      <c r="D12" t="n">
+        <v>2</v>
+      </c>
+      <c r="E12" t="n">
+        <v>8</v>
+      </c>
+      <c r="F12" t="n">
+        <v>4</v>
+      </c>
+      <c r="G12" t="n">
+        <v>1.444110928103328</v>
+      </c>
+      <c r="H12" t="n">
+        <v>141116</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>11</v>
+      </c>
+      <c r="B13" t="n">
+        <v>100000000</v>
+      </c>
+      <c r="C13" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D13" t="n">
+        <v>2</v>
+      </c>
+      <c r="E13" t="n">
+        <v>8</v>
+      </c>
+      <c r="F13" t="n">
+        <v>4</v>
+      </c>
+      <c r="G13" t="n">
+        <v>1.40458363853395</v>
+      </c>
+      <c r="H13" t="n">
+        <v>141776</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>12</v>
+      </c>
+      <c r="B14" t="n">
+        <v>100000000</v>
+      </c>
+      <c r="C14" t="n">
+        <v>10</v>
+      </c>
+      <c r="D14" t="n">
+        <v>2</v>
+      </c>
+      <c r="E14" t="n">
+        <v>16</v>
+      </c>
+      <c r="F14" t="n">
+        <v>8</v>
+      </c>
+      <c r="G14" t="n">
+        <v>1.463829785585403</v>
+      </c>
+      <c r="H14" t="n">
+        <v>140732</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>13</v>
+      </c>
+      <c r="B15" t="n">
+        <v>100000000</v>
+      </c>
+      <c r="C15" t="n">
+        <v>100</v>
+      </c>
+      <c r="D15" t="n">
+        <v>2</v>
+      </c>
+      <c r="E15" t="n">
+        <v>16</v>
+      </c>
+      <c r="F15" t="n">
+        <v>8</v>
+      </c>
+      <c r="G15" t="n">
+        <v>1.434639092534781</v>
+      </c>
+      <c r="H15" t="n">
+        <v>141416</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>14</v>
+      </c>
+      <c r="B16" t="n">
+        <v>100000000</v>
+      </c>
+      <c r="C16" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D16" t="n">
+        <v>2</v>
+      </c>
+      <c r="E16" t="n">
+        <v>16</v>
+      </c>
+      <c r="F16" t="n">
+        <v>8</v>
+      </c>
+      <c r="G16" t="n">
+        <v>1.358143012970686</v>
+      </c>
+      <c r="H16" t="n">
+        <v>141264</v>
       </c>
     </row>
   </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="B1:H1"/>
-  </ignoredErrors>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update from Ganymede2 run
</commit_message>
<xml_diff>
--- a/phys5v48hw/hw4/output/asyncLorentz/asyncLorentzCat.xlsx
+++ b/phys5v48hw/hw4/output/asyncLorentz/asyncLorentzCat.xlsx
@@ -1,79 +1,3 @@
-
-<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <workbookPr codeName="ThisWorkbook"/>
-  <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-  </sheets>
-</workbook>
-</file>
-
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
-</file>
-
-<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
-  <fonts count="1">
-    <font>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-  </fonts>
-  <fills count="2">
-    <fill>
-      <patternFill patternType="none"/>
-    </fill>
-    <fill>
-      <patternFill patternType="gray125"/>
-    </fill>
-  </fills>
-  <borders count="1">
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-  </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-  </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-  </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
-  </cellStyles>
-  <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
-</styleSheet>
-</file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
@@ -150,7 +74,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -185,7 +108,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -220,16 +142,20 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="100000"/>
-                <a:shade val="100000"/>
+                <a:shade val="51000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-                <a:shade val="100000"/>
-                <a:satMod val="350000"/>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -351,80 +277,7 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults>
-    <a:spDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="3">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="lt1"/>
-        </a:fontRef>
-      </a:style>
-    </a:spDef>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
+  <a:objectDefaults/>
   <a:extraClrSchemeLst/>
 </a:theme>
-</file>
-
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="B1:H1"/>
-  <sheetData>
-    <row r="1">
-      <c r="B1" t="str">
-        <v>Problem Size (n)</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Bins</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Nodes</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Ranks</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Threads Per Rank</v>
-      </c>
-      <c r="G1" t="str">
-        <v>Runtime</v>
-      </c>
-      <c r="H1" t="str">
-        <v>Peak Memory</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="B1:H1"/>
-  </ignoredErrors>
-</worksheet>
 </file>
</xml_diff>